<commit_message>
Remove Seasoning and quantity in ShoppingList
</commit_message>
<xml_diff>
--- a/db/Db_ddl & examples.xlsx
+++ b/db/Db_ddl & examples.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Beaming\Desktop\Database\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Beaming\Desktop\TeamSEM_b20_Project\db\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA4D7A3B-BF4A-43AF-B995-B95A0572D659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BB3BAA3-CFC3-4633-BF8E-81B12944FA97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="765" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="765" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Recipe" sheetId="1" r:id="rId1"/>
@@ -18,10 +18,8 @@
     <sheet name="Recipe_Ingredient" sheetId="3" r:id="rId3"/>
     <sheet name="Tag" sheetId="4" r:id="rId4"/>
     <sheet name="Recipe_Tag" sheetId="5" r:id="rId5"/>
-    <sheet name="Seasoning" sheetId="8" r:id="rId6"/>
-    <sheet name="Recipe_Seasoning" sheetId="9" r:id="rId7"/>
-    <sheet name="MealPlan" sheetId="6" r:id="rId8"/>
-    <sheet name="ShoppingList" sheetId="7" r:id="rId9"/>
+    <sheet name="MealPlan" sheetId="6" r:id="rId6"/>
+    <sheet name="ShoppingList" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -33,15 +31,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="41">
   <si>
     <t>recipeID</t>
-  </si>
-  <si>
-    <t>unit</t>
-  </si>
-  <si>
-    <t>lb</t>
   </si>
   <si>
     <t>broccli</t>
@@ -208,40 +200,10 @@
     <t>ingreID</t>
   </si>
   <si>
-    <t>sID</t>
-  </si>
-  <si>
-    <t>seasoning</t>
-  </si>
-  <si>
-    <t>salt</t>
-  </si>
-  <si>
-    <t>pepper</t>
-  </si>
-  <si>
-    <t>soy source</t>
-  </si>
-  <si>
-    <t>some</t>
-  </si>
-  <si>
-    <t>pinch</t>
-  </si>
-  <si>
     <t>qty(NUMERIC type, default =1)</t>
   </si>
   <si>
-    <t>qty(text type, default =null)</t>
-  </si>
-  <si>
-    <t>qty(NUMERIC type)</t>
-  </si>
-  <si>
     <t>title(default not null)</t>
-  </si>
-  <si>
-    <t>sID (composite key)</t>
   </si>
   <si>
     <t>wID (DATE type)</t>
@@ -288,10 +250,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -584,22 +547,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B1" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="C1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E1" t="s">
         <v>21</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>22</v>
-      </c>
-      <c r="E1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F1" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -607,19 +570,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>6</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>7</v>
-      </c>
-      <c r="E2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -627,10 +590,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -649,10 +612,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -660,7 +623,7 @@
         <v>101</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -668,7 +631,7 @@
         <v>102</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -691,13 +654,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C1" t="s">
         <v>38</v>
       </c>
-      <c r="C1" t="s">
-        <v>47</v>
-      </c>
       <c r="D1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -711,7 +674,7 @@
         <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -733,7 +696,7 @@
         <v>5</v>
       </c>
       <c r="D4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -747,7 +710,7 @@
         <v>5</v>
       </c>
       <c r="D5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -766,10 +729,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -777,7 +740,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -785,7 +748,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -793,7 +756,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -814,7 +777,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -839,102 +802,6 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F0620F2-D1D7-47E1-A83E-4B8A6CD5E077}">
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>44</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F9C75C5-6185-46BA-9642-462962A2970A}">
-  <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="22.21875" customWidth="1"/>
-    <col min="3" max="3" width="24.77734375" customWidth="1"/>
-    <col min="4" max="4" width="16.6640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="C1" t="s">
-        <v>48</v>
-      </c>
-      <c r="D1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>1</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0448313F-88A5-4ADC-9AF1-6DA2EB3B2C0C}">
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -945,16 +812,16 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B1" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="C1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E1" t="s">
         <v>0</v>
@@ -968,10 +835,10 @@
         <v>46097</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E2">
         <v>2</v>
@@ -985,10 +852,10 @@
         <v>46097</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -1002,10 +869,10 @@
         <v>46097</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E4">
         <v>2</v>
@@ -1017,80 +884,70 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97D32EFC-032C-4779-B542-0757EFFBECAF}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.44140625" customWidth="1"/>
-    <col min="2" max="2" width="9" customWidth="1"/>
-    <col min="4" max="4" width="17.21875" customWidth="1"/>
-    <col min="5" max="5" width="19.33203125" customWidth="1"/>
+    <col min="1" max="2" width="10.44140625" customWidth="1"/>
+    <col min="3" max="3" width="9" customWidth="1"/>
+    <col min="4" max="4" width="19.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B1" t="s">
-        <v>39</v>
+        <v>26</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="D1" t="s">
-        <v>49</v>
-      </c>
-      <c r="E1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
         <v>101</v>
       </c>
-      <c r="C2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
         <v>102</v>
       </c>
-      <c r="D3">
-        <v>4</v>
-      </c>
-      <c r="E3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4">
         <v>101</v>
       </c>
-      <c r="C4" t="s">
-        <v>33</v>
-      </c>
-      <c r="D4">
-        <v>2</v>
-      </c>
-      <c r="E4" t="s">
-        <v>6</v>
+      <c r="D4" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor: Add 'input_item' to ShoppingList; Merge 'qty' and 'unit' in Ingredient into one column 'amount'
</commit_message>
<xml_diff>
--- a/db/Db_ddl & examples.xlsx
+++ b/db/Db_ddl & examples.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Beaming\Desktop\TeamSEM_b20_Project\db\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BB3BAA3-CFC3-4633-BF8E-81B12944FA97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82058E16-00E9-4EA4-96CF-207FAF5F5D51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="765" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="765" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Recipe" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="42">
   <si>
     <t>recipeID</t>
   </si>
@@ -72,9 +72,6 @@
     <t>day</t>
   </si>
   <si>
-    <t>mealTime</t>
-  </si>
-  <si>
     <t>Monday</t>
   </si>
   <si>
@@ -87,19 +84,7 @@
     <t>Lunch</t>
   </si>
   <si>
-    <t>unit(default = null)</t>
-  </si>
-  <si>
     <t>favorites(default = no)</t>
-  </si>
-  <si>
-    <t>cook_time(default=null)</t>
-  </si>
-  <si>
-    <t>instructions(default = null)</t>
-  </si>
-  <si>
-    <t>image(default=null)</t>
   </si>
   <si>
     <r>
@@ -179,12 +164,6 @@
     <t>tag (unique)</t>
   </si>
   <si>
-    <t>oz</t>
-  </si>
-  <si>
-    <t>lbs</t>
-  </si>
-  <si>
     <t>Steak</t>
   </si>
   <si>
@@ -200,13 +179,37 @@
     <t>ingreID</t>
   </si>
   <si>
-    <t>qty(NUMERIC type, default =1)</t>
-  </si>
-  <si>
     <t>title(default not null)</t>
   </si>
   <si>
     <t>wID (DATE type)</t>
+  </si>
+  <si>
+    <t>input_item</t>
+  </si>
+  <si>
+    <t>broconni</t>
+  </si>
+  <si>
+    <t>amount</t>
+  </si>
+  <si>
+    <t>5 lbs</t>
+  </si>
+  <si>
+    <t>5 oz</t>
+  </si>
+  <si>
+    <t>cook_time</t>
+  </si>
+  <si>
+    <t>instructions</t>
+  </si>
+  <si>
+    <t>image</t>
+  </si>
+  <si>
+    <t>meal_type</t>
   </si>
 </sst>
 </file>
@@ -250,11 +253,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -547,22 +549,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E1" t="s">
-        <v>21</v>
-      </c>
       <c r="F1" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -590,10 +592,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="D3" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -612,10 +614,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="B1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -641,7 +643,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77485178-4EDD-4D2D-9CBD-13B22AED9FB2}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="34.109375" customWidth="1"/>
@@ -649,35 +651,29 @@
     <col min="4" max="4" width="17.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="C1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2">
         <v>101</v>
       </c>
-      <c r="C2">
-        <v>5</v>
-      </c>
-      <c r="D2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -685,32 +681,26 @@
         <v>102</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4">
         <v>101</v>
       </c>
-      <c r="C4">
-        <v>5</v>
-      </c>
-      <c r="D4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>3</v>
       </c>
       <c r="B5">
         <v>101</v>
       </c>
-      <c r="C5">
-        <v>5</v>
-      </c>
-      <c r="D5" t="s">
-        <v>32</v>
+      <c r="C5" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -732,7 +722,7 @@
         <v>8</v>
       </c>
       <c r="B1" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -777,7 +767,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -808,20 +798,21 @@
   <cols>
     <col min="1" max="1" width="9.44140625" customWidth="1"/>
     <col min="2" max="2" width="13.6640625" customWidth="1"/>
+    <col min="4" max="4" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="B1" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="C1" t="s">
         <v>12</v>
       </c>
       <c r="D1" t="s">
-        <v>13</v>
+        <v>41</v>
       </c>
       <c r="E1" t="s">
         <v>0</v>
@@ -835,10 +826,10 @@
         <v>46097</v>
       </c>
       <c r="C2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" t="s">
         <v>14</v>
-      </c>
-      <c r="D2" t="s">
-        <v>15</v>
       </c>
       <c r="E2">
         <v>2</v>
@@ -852,10 +843,10 @@
         <v>46097</v>
       </c>
       <c r="C3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" t="s">
         <v>16</v>
-      </c>
-      <c r="D3" t="s">
-        <v>17</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -869,10 +860,10 @@
         <v>46097</v>
       </c>
       <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" t="s">
         <v>14</v>
-      </c>
-      <c r="D4" t="s">
-        <v>15</v>
       </c>
       <c r="E4">
         <v>2</v>
@@ -886,29 +877,33 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97D32EFC-032C-4779-B542-0757EFFBECAF}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="10.44140625" customWidth="1"/>
     <col min="3" max="3" width="9" customWidth="1"/>
-    <col min="4" max="4" width="19.33203125" customWidth="1"/>
+    <col min="4" max="4" width="10.6640625" customWidth="1"/>
+    <col min="5" max="5" width="19.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B1" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="D1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+      <c r="E1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -918,11 +913,11 @@
       <c r="C2">
         <v>101</v>
       </c>
-      <c r="D2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -932,11 +927,11 @@
       <c r="C3">
         <v>102</v>
       </c>
-      <c r="D3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -946,8 +941,16 @@
       <c r="C4">
         <v>101</v>
       </c>
-      <c r="D4" t="s">
-        <v>25</v>
+      <c r="E4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="D5" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>